<commit_message>
aun no se ve bien el arbol
</commit_message>
<xml_diff>
--- a/actions/corpus/palabras.xlsx
+++ b/actions/corpus/palabras.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E80"/>
+  <dimension ref="A1:E86"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="12.63" customWidth="1" style="9" min="1" max="2"/>
@@ -811,12 +811,12 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>xoo</t>
+          <t>yankon</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t>Corregido por validador Corrección validador: verde yankon → xoo (verde y azul son distintos en shipibo; ya no comparten forma).</t>
+          <t>Corregido por validador</t>
         </is>
       </c>
     </row>
@@ -1683,61 +1683,71 @@
     <row r="67" ht="15.75" customHeight="1" s="9">
       <c r="A67" s="0" t="inlineStr">
         <is>
-          <t>per_001</t>
+          <t>ani_014</t>
         </is>
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>hombre</t>
+          <t>tigre</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
         <is>
-          <t>joni</t>
+          <t>sere ino</t>
         </is>
       </c>
       <c r="E67" s="0" t="inlineStr">
         <is>
-          <t>PROPUESTA cuentos - validar con hablante</t>
+          <t>PROPUESTA cuentos - validar con hablante Corrección validador (retro): ino → sere ino.</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15.75" customHeight="1" s="9">
       <c r="A68" s="0" t="inlineStr">
         <is>
-          <t>per_002</t>
+          <t>ani_015</t>
         </is>
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>cuñado</t>
+          <t>motelo</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
         <is>
-          <t>chai</t>
+          <t>manan xawe</t>
+        </is>
+      </c>
+      <c r="D68" s="0" t="inlineStr">
+        <is>
+          <t>tortuga terrestre</t>
         </is>
       </c>
       <c r="E68" s="0" t="inlineStr">
         <is>
-          <t>PROPUESTA cuentos - validar con hablante</t>
+          <t>PROPUESTA cuentos - validar con hablante Corrección validador (retro): mananxawe → manan xawe.</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15.75" customHeight="1" s="9">
       <c r="A69" s="0" t="inlineStr">
         <is>
-          <t>per_003</t>
+          <t>ani_016</t>
         </is>
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>madre</t>
+          <t>paujil</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
         <is>
-          <t>tita</t>
+          <t>jasin</t>
+        </is>
+      </c>
+      <c r="D69" s="0" t="inlineStr">
+        <is>
+          <t>ave de la selva</t>
         </is>
       </c>
       <c r="E69" s="0" t="inlineStr">
@@ -1749,17 +1759,22 @@
     <row r="70" ht="15.75" customHeight="1" s="9">
       <c r="A70" s="0" t="inlineStr">
         <is>
-          <t>per_004</t>
+          <t>ani_017</t>
         </is>
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t>señorita</t>
+          <t>camungo</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
         <is>
-          <t>xontako</t>
+          <t>abokoma</t>
+        </is>
+      </c>
+      <c r="D70" s="0" t="inlineStr">
+        <is>
+          <t>ave</t>
         </is>
       </c>
       <c r="E70" s="0" t="inlineStr">
@@ -1771,17 +1786,17 @@
     <row r="71" ht="15.75" customHeight="1" s="9">
       <c r="A71" s="0" t="inlineStr">
         <is>
-          <t>per_005</t>
+          <t>ani_018</t>
         </is>
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t>hijos</t>
+          <t>zorro</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
         <is>
-          <t>bakebo</t>
+          <t>maxo</t>
         </is>
       </c>
       <c r="E71" s="0" t="inlineStr">
@@ -1793,232 +1808,338 @@
     <row r="72" ht="15.75" customHeight="1" s="9">
       <c r="A72" s="0" t="inlineStr">
         <is>
-          <t>ani_014</t>
+          <t>ani_019</t>
         </is>
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>tigre</t>
+          <t>loro</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
         <is>
-          <t>sere ino</t>
+          <t>bawa</t>
         </is>
       </c>
       <c r="E72" s="0" t="inlineStr">
         <is>
-          <t>PROPUESTA cuentos - validar con hablante Corrección validador (retro): ino → sere ino.</t>
+          <t>PROPUESTA cuentos - validar con hablante</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15.75" customHeight="1" s="9">
       <c r="A73" s="0" t="inlineStr">
         <is>
-          <t>ani_015</t>
+          <t>nat_012</t>
         </is>
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t>motelo</t>
+          <t>cocha</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
         <is>
-          <t>manan xawe</t>
+          <t>ian</t>
         </is>
       </c>
       <c r="D73" s="0" t="inlineStr">
         <is>
-          <t>tortuga terrestre</t>
+          <t>laguna</t>
         </is>
       </c>
       <c r="E73" s="0" t="inlineStr">
         <is>
-          <t>PROPUESTA cuentos - validar con hablante Corrección validador (retro): mananxawe → manan xawe.</t>
+          <t>PROPUESTA cuentos - validar con hablante</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15.75" customHeight="1" s="9">
-      <c r="A74" s="0" t="inlineStr">
-        <is>
-          <t>ani_016</t>
-        </is>
-      </c>
-      <c r="B74" s="0" t="inlineStr">
-        <is>
-          <t>paujil</t>
-        </is>
-      </c>
-      <c r="C74" s="0" t="inlineStr">
-        <is>
-          <t>jasin</t>
-        </is>
-      </c>
-      <c r="D74" s="0" t="inlineStr">
-        <is>
-          <t>ave de la selva</t>
-        </is>
-      </c>
-      <c r="E74" s="0" t="inlineStr">
-        <is>
-          <t>PROPUESTA cuentos - validar con hablante</t>
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>fam_001</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>mamá</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>tita</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Categoría familia (reemplaza a personas). Aportado por validador.</t>
         </is>
       </c>
     </row>
     <row r="75" ht="15.75" customHeight="1" s="9">
-      <c r="A75" s="0" t="inlineStr">
-        <is>
-          <t>ani_017</t>
-        </is>
-      </c>
-      <c r="B75" s="0" t="inlineStr">
-        <is>
-          <t>camungo</t>
-        </is>
-      </c>
-      <c r="C75" s="0" t="inlineStr">
-        <is>
-          <t>abokoma</t>
-        </is>
-      </c>
-      <c r="D75" s="0" t="inlineStr">
-        <is>
-          <t>ave</t>
-        </is>
-      </c>
-      <c r="E75" s="0" t="inlineStr">
-        <is>
-          <t>PROPUESTA cuentos - validar con hablante</t>
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>fam_002</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>papá</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>papa</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Categoría familia (reemplaza a personas). Aportado por validador.</t>
         </is>
       </c>
     </row>
     <row r="76" ht="15.75" customHeight="1" s="9">
-      <c r="A76" s="0" t="inlineStr">
-        <is>
-          <t>ani_018</t>
-        </is>
-      </c>
-      <c r="B76" s="0" t="inlineStr">
-        <is>
-          <t>zorro</t>
-        </is>
-      </c>
-      <c r="C76" s="0" t="inlineStr">
-        <is>
-          <t>maxo</t>
-        </is>
-      </c>
-      <c r="E76" s="0" t="inlineStr">
-        <is>
-          <t>PROPUESTA cuentos - validar con hablante</t>
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>fam_003</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>hija</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>ainbo bake</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Categoría familia (reemplaza a personas). Aportado por validador.</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15.75" customHeight="1" s="9">
-      <c r="A77" s="0" t="inlineStr">
-        <is>
-          <t>ani_019</t>
-        </is>
-      </c>
-      <c r="B77" s="0" t="inlineStr">
-        <is>
-          <t>loro</t>
-        </is>
-      </c>
-      <c r="C77" s="0" t="inlineStr">
-        <is>
-          <t>bawa</t>
-        </is>
-      </c>
-      <c r="E77" s="0" t="inlineStr">
-        <is>
-          <t>PROPUESTA cuentos - validar con hablante</t>
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>fam_004</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>hijo</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>benbo bake</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Categoría familia (reemplaza a personas). Aportado por validador.</t>
         </is>
       </c>
     </row>
     <row r="78" ht="15.75" customHeight="1" s="9">
-      <c r="A78" s="0" t="inlineStr">
-        <is>
-          <t>nat_012</t>
-        </is>
-      </c>
-      <c r="B78" s="0" t="inlineStr">
-        <is>
-          <t>cocha</t>
-        </is>
-      </c>
-      <c r="C78" s="0" t="inlineStr">
-        <is>
-          <t>ian</t>
-        </is>
-      </c>
-      <c r="D78" s="0" t="inlineStr">
-        <is>
-          <t>laguna</t>
-        </is>
-      </c>
-      <c r="E78" s="0" t="inlineStr">
-        <is>
-          <t>PROPUESTA cuentos - validar con hablante</t>
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>fam_005</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>bebé</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>binshin</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Categoría familia (reemplaza a personas). Aportado por validador.</t>
         </is>
       </c>
     </row>
     <row r="79" ht="15.75" customHeight="1" s="9">
-      <c r="A79" s="0" t="inlineStr">
-        <is>
-          <t>obj_010</t>
-        </is>
-      </c>
-      <c r="B79" s="0" t="inlineStr">
-        <is>
-          <t>masato</t>
-        </is>
-      </c>
-      <c r="C79" s="0" t="inlineStr">
-        <is>
-          <t>atsa xeati</t>
-        </is>
-      </c>
-      <c r="D79" s="0" t="inlineStr">
-        <is>
-          <t>bebida de yuca</t>
-        </is>
-      </c>
-      <c r="E79" s="0" t="inlineStr">
-        <is>
-          <t>PROPUESTA cuentos - validar con hablante | Corregido por validador</t>
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>fam_006</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>abuela</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>yoxan</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Categoría familia (reemplaza a personas). Aportado por validador.</t>
         </is>
       </c>
     </row>
     <row r="80" ht="15.75" customHeight="1" s="9">
-      <c r="A80" s="0" t="inlineStr">
-        <is>
-          <t>obj_011</t>
-        </is>
-      </c>
-      <c r="B80" s="0" t="inlineStr">
-        <is>
-          <t>fiesta</t>
-        </is>
-      </c>
-      <c r="C80" s="0" t="inlineStr">
-        <is>
-          <t>pishta</t>
-        </is>
-      </c>
-      <c r="E80" s="0" t="inlineStr">
-        <is>
-          <t>PROPUESTA cuentos - validar con hablante</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="15.75" customHeight="1" s="9"/>
-    <row r="82" ht="15.75" customHeight="1" s="9"/>
-    <row r="83" ht="15.75" customHeight="1" s="9"/>
-    <row r="84" ht="15.75" customHeight="1" s="9"/>
-    <row r="85" ht="15.75" customHeight="1" s="9"/>
-    <row r="86" ht="15.75" customHeight="1" s="9"/>
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>fam_007</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>abuelo</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>yosi</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Categoría familia (reemplaza a personas). Aportado por validador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="15.75" customHeight="1" s="9">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>fam_008</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>nieto</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>baba</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Categoría familia (reemplaza a personas). Aportado por validador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="15.75" customHeight="1" s="9">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>fam_009</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>tío</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>koka</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Categoría familia (reemplaza a personas). Aportado por validador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="15.75" customHeight="1" s="9">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>fam_010</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>tía</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>wata</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Categoría familia (reemplaza a personas). Aportado por validador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="15.75" customHeight="1" s="9">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>fam_011</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>primo</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>wetsa</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Categoría familia (reemplaza a personas). Aportado por validador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="15.75" customHeight="1" s="9">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>fam_012</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>hermano</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>wetsako</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Categoría familia (reemplaza a personas). Aportado por validador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="15.75" customHeight="1" s="9">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>fam_013</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>hermana</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>wetsa</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Categoría familia (reemplaza a personas). Aportado por validador.</t>
+        </is>
+      </c>
+    </row>
     <row r="87" ht="15.75" customHeight="1" s="9"/>
     <row r="88" ht="15.75" customHeight="1" s="9"/>
     <row r="89" ht="15.75" customHeight="1" s="9"/>

</xml_diff>